<commit_message>
Fix CRM demo: filter institutional investors, cap portfolio at 15
Tightened exclusion filters for securitization vehicles (BORROWER,
PORTFOLIO, CONREX, SFR PROPERTY, etc.), builder entities, and
limited partnerships. Capped at 15 properties to exclude
institutional-scale portfolios. Brand color updated to #366F78.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sales/demo_tearsheets/demo_crm_northside.xlsx
+++ b/sales/demo_tearsheets/demo_crm_northside.xlsx
@@ -62,8 +62,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00008080"/>
-        <bgColor rgb="00008080"/>
+        <fgColor rgb="00366F78"/>
+        <bgColor rgb="00366F78"/>
       </patternFill>
     </fill>
     <fill>
@@ -557,15 +557,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MFREVF V - ASTER LP LIMITED PARTNERSHIP</t>
+          <t>LANGER, LENA TRUSTEE LANGER, OLEG TRUSTEE</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cary</t>
+          <t>Garner, Knightdale</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>$24.0M</t>
+          <t>$1.7M</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -605,15 +605,15 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>DOORS HOLDINGS 2024 LLC</t>
+          <t>VM PRONTO LLC</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Knightdale, Raleigh</t>
+          <t>Fuquay-Varina, Garner, Raleigh</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -636,12 +636,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>$3.5M</t>
+          <t>$1.8M</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -653,15 +653,15 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LANGER, LENA TRUSTEE LANGER, OLEG TRUSTEE</t>
+          <t>H&amp;H CONSTRUCTORS OF FAYETTEVILLE LLC</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Garner, Knightdale</t>
+          <t>Cary, Wake Forest</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -679,12 +679,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>$1.7M</t>
+          <t>$4.2M</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -701,15 +701,15 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>NC EDWARDS MILL LLC BS TOWNHOMES LLC</t>
+          <t>WU, CLARISSA QING TRUSTEE WANG, YIBING TRUSTEE</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Cary, Garner, Raleigh</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -732,12 +732,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>$8.1M</t>
+          <t>$1.4M</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2022-04</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -749,15 +749,15 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ARMM ASSETS 3 LLC</t>
+          <t>MJ RENTAL I LLC</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Knightdale, Raleigh, Wendell</t>
+          <t>Garner, Raleigh</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -780,12 +780,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>$1.5M</t>
+          <t>$2.5M</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2018-09</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -797,11 +797,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>VB BC LLC</t>
+          <t>TWO CAT INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -828,12 +828,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>$15.6M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2016-06</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -845,15 +845,15 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TOLL SOUTHEAST LP COMPANY INC</t>
+          <t>MISRA, AKHILESH TRUSTEE AKHILESH MISRA LIVING TRUST</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Apex, Garner, Holly Springs, Knightdale, Raleigh</t>
+          <t>Cary, Fuquay-Varina, Holly Springs</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -876,12 +876,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>$11.4M</t>
+          <t>$2.2M</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2017-06</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -893,15 +893,15 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ARMM ASSET COMPANY 2 LLC</t>
+          <t>VESTED REALTY LLC</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Knightdale, Raleigh</t>
+          <t>Raleigh, Rolesville</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -924,12 +924,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>$1.9M</t>
+          <t>$2.0M</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2022-06</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -941,15 +941,15 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>OP SPE SUMMIT LLC</t>
+          <t>HARRINGTON GROVE HOLDINGS LLC</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Cary, Fuquay-Varina, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -977,7 +977,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2021-06</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -989,15 +989,15 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>FLI WW SFR 1 LLC</t>
+          <t>APOSTLE INC</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Cary</t>
+          <t>Fuquay-Varina, Garner, Raleigh, Rolesville</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
@@ -1020,12 +1020,12 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>$19.9M</t>
+          <t>$5.0M</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1037,15 +1037,15 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>OP SPE PHX1 LLC</t>
+          <t>KL LB BUY 3 LLC</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Cary, Raleigh, Wendell</t>
+          <t>Apex</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>$2.3M</t>
+          <t>$10.2M</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1085,15 +1085,15 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>PURCHASING FUND 2025-1 LLC</t>
+          <t>CANNON NC RENTALS III LLC</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Cary, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>$1.8M</t>
+          <t>$2.8M</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2016-07</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1133,15 +1133,15 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PURCHASING FUND 2023-2 LLC</t>
+          <t>NOBLE-CARBAJAL, MELADEE TRUSTEE MELADEE NOBLE 2019 TRUST</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Apex, Cary, Fuquay-Varina, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>$4.8M</t>
+          <t>$909K</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2020-08</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1181,15 +1181,15 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>VM PRONTO LLC</t>
+          <t>THE TRUST OF BOONE WAKE COUNTY NORTH CAROLINA WCNC</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
@@ -1207,17 +1207,17 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>$1.8M</t>
+          <t>$2.4M</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -1229,15 +1229,15 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FREO PROGRESS LLC</t>
+          <t>RXR LEN APEX OWNER LLC</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh</t>
+          <t>Apex</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>$1.0M</t>
+          <t>$3.3M</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1277,15 +1277,15 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>DOORS HOLDINGS 2025-1 LLC</t>
+          <t>ARAZI, VICTOR COHEN TRUSTEE COHEN, LAURA TRUSTEE</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wendell</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -1308,12 +1308,12 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>$3.9M</t>
+          <t>$1.6M</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2019-07</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -1325,15 +1325,15 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DOORS HOLDINGS 2025-2 LLC</t>
+          <t>RS RENTAL III-B LLC</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wendell</t>
+          <t>Raleigh, Wake Forest, Wendell</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1356,12 +1356,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>$4.0M</t>
+          <t>$4.3M</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1373,15 +1373,15 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>H &amp; H CONSTRUCTORS OF FAYETTEVILLE LLC</t>
+          <t>LEBLANC PROPERTY HOLDINGS LLC</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>89</v>
+        <v>5</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Knightdale</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
@@ -1404,12 +1404,12 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>$37.1M</t>
+          <t>$1.3M</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2019-09</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -1421,15 +1421,15 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>H&amp;H CONSTRUCTORS OF FAYETTEVILLE LLC</t>
+          <t>THE CIANO FAMILY TRUST</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Cary, Wake Forest</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1447,17 +1447,17 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>$4.2M</t>
+          <t>$1.4M</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2021-06</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1469,15 +1469,15 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>HUDSON SFR PROPERTY HOLDINGS II LLC</t>
+          <t>BAF 4 LLC</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Holly Springs, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>$9.5M</t>
+          <t>$2.4M</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2021-05</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -1517,15 +1517,15 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CANNON NC RENTALS II LLC</t>
+          <t>BBRK LLC</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Apex, Cary, Holly Springs, Raleigh</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>$3.3M</t>
+          <t>$2.6M</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2020-05</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1565,15 +1565,15 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>RH EVERGREEN OWNERCO LLC</t>
+          <t>CANNON NC RENTALS LLC</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Knightdale, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1596,12 +1596,12 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>$957K</t>
+          <t>$2.8M</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>2020-12</t>
+          <t>2020-11</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1613,15 +1613,15 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MILE HIGH TL BORROWER 1 (CORE) LLC</t>
+          <t>PATRIOT CANYON PROPERTIES LLC</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1644,12 +1644,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>$3.1M</t>
+          <t>$1.7M</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2021-06</t>
+          <t>2016-06</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1661,7 +1661,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>TWO CAT INVESTMENTS LLC</t>
+          <t>STAGE II PROPERTIES LLC</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Garner, Raleigh, Wendell</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1692,12 +1692,12 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>$1.1M</t>
+          <t>$1.9M</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>2016-06</t>
+          <t>2017-08</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -1709,15 +1709,15 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MILE HIGH BORROWER 1 (VALUE) LLC</t>
+          <t>GOLDBEAR INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Holly Springs, Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Cary, Raleigh</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1740,12 +1740,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>$6.1M</t>
+          <t>$2.4M</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2022-06</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1757,11 +1757,11 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>CANNON NC LLC</t>
+          <t>MOLLOY ENTERPRISES LLC</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>$3.5M</t>
+          <t>$1.6M</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>2017-04</t>
+          <t>2018-11</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -1805,15 +1805,15 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>WINDSOR CREST PROPERTIES INC</t>
+          <t>SAS INSTITUTE INC</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Cary</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>$12.3M</t>
+          <t>$1.4M</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2003-06</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -1853,15 +1853,15 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>MILE HIGH TL BORROWER 1 (INCOME) LLC</t>
+          <t>RIGHT FORCE INC</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Holly Springs, Knightdale, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1879,17 +1879,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>$7.1M</t>
+          <t>$4.3M</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>2021-10</t>
+          <t>2009-08</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -1901,15 +1901,15 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AMH 2014-2 BORROWER LLC</t>
+          <t>ZOOMZ INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>176</v>
+        <v>4</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Rolesville, Wake Forest, Wendell</t>
+          <t>Apex, Fuquay-Varina, Wendell</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1932,12 +1932,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>$63.4M</t>
+          <t>$1.5M</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>2014-03</t>
+          <t>2021-05</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -1949,15 +1949,15 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>WU, CLARISSA QING TRUSTEE WANG, YIBING TRUSTEE</t>
+          <t>21 JUMPSTREET LLC</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Cary, Garner, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1980,12 +1980,12 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>$1.4M</t>
+          <t>$1.7M</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>2022-04</t>
+          <t>2012-11</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -1997,11 +1997,11 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AC BLACKWOLF RUN OWNER LLC</t>
+          <t>VOGLER, JAMES BREVARD III TRUSTEE LINDEN, SARAH SKYE TRUSTEE</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>329</v>
+        <v>6</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -2028,12 +2028,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>$80.9M</t>
+          <t>$2.0M</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2015-11</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2045,15 +2045,15 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>BAF ASSETS 3 LLC</t>
+          <t>AMH NC PROPERTIES, L.P.</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Rolesville, Wake Forest</t>
+          <t>Fuquay-Varina, Raleigh, Rolesville, Wake Forest</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2076,12 +2076,12 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>$6.5M</t>
+          <t>$3.4M</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>2021-02</t>
+          <t>2018-02</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -2093,15 +2093,15 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CONREX ML PORTFOLIO 2019-01 OPERATING COMPANY, LLC</t>
+          <t>AMH ROMAN TWO NC LLC</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Garner, Wendell</t>
+          <t>Apex, Cary, Fuquay-Varina, Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>$603K</t>
+          <t>$5.9M</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>2018-09</t>
+          <t>2016-03</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2141,15 +2141,15 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>GRANTHAM HOLDINGS LLC</t>
+          <t>CANNON NC LLC</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2172,12 +2172,12 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>$2.1M</t>
+          <t>$3.5M</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>2010-10</t>
+          <t>2017-04</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2189,7 +2189,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CANNON NC RENTALS III LLC</t>
+          <t>SCHWARTZ, JEFFREY TRUSTEE BARRY, CYNTHIA TRUSTEE</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>$2.8M</t>
+          <t>$3.1M</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>2016-07</t>
+          <t>2016-05</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2237,15 +2237,15 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BAF ASSETS 4 LLC</t>
+          <t>DIVERSIFIED RESIDENTIAL HOMES 1 LLC</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Garner, Raleigh, Wendell</t>
+          <t>Knightdale, Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>$1.6M</t>
+          <t>$2.6M</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>2021-08</t>
+          <t>2021-11</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2285,15 +2285,15 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GOLDBEAR INVESTMENTS LLC</t>
+          <t>RH EVERGREEN OWNERCO LLC</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Cary, Raleigh</t>
+          <t>Knightdale, Raleigh</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2316,12 +2316,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>$2.4M</t>
+          <t>$957K</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2020-12</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2333,15 +2333,15 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>ARAZI, VICTOR COHEN TRUSTEE COHEN, LAURA TRUSTEE</t>
+          <t>CANNON NC RENTALS II LLC</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2364,12 +2364,12 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>$1.6M</t>
+          <t>$3.3M</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>2019-07</t>
+          <t>2021-09</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -2381,15 +2381,15 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MISRA, AKHILESH TRUSTEE AKHILESH MISRA LIVING TRUST</t>
+          <t>GRANTHAM HOLDINGS LLC</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Cary, Fuquay-Varina, Holly Springs</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2412,12 +2412,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>$2.2M</t>
+          <t>$2.1M</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2017-06</t>
+          <t>2010-10</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2429,15 +2429,15 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>PMC SFR BORROWER LLC</t>
+          <t>HEBERT, ERIC TRUSTEE THE ERIC HEBERT FAMILY TRUST</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Garner, Holly Springs, Knightdale, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2460,12 +2460,12 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>$3.1M</t>
+          <t>$3.4M</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>2017-10</t>
+          <t>2016-12</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -2477,11 +2477,11 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>RIGHT FORCE INC</t>
+          <t>NGP INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2503,17 +2503,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>$4.3M</t>
+          <t>$1.7M</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>2009-08</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2525,15 +2525,15 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>LEBLANC PROPERTY HOLDINGS LLC</t>
+          <t>FALCOCCHIA, EDDIE TRUSTEE 2003 EDDIE FALCOCCHIA REVOCABLE LIVING TRUST</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Cary, Raleigh</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
@@ -2556,14 +2556,10 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>$1.3M</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>2019-09</t>
-        </is>
-      </c>
+          <t>$2.4M</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2573,15 +2569,15 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BAF 4 LLC</t>
+          <t>GVII-RS OWNERCO LLC</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2590,7 +2586,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2604,12 +2600,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>$2.4M</t>
+          <t>$1.4M</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>2021-05</t>
+          <t>2022-09</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2621,24 +2617,24 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>MERMAID BORROWER LLC</t>
+          <t>FIDLER, VAN A TRUSTEE FIDLER, REGINA E TRUSTEE</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Raleigh, Rolesville, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
@@ -2652,12 +2648,12 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>$2.8M</t>
+          <t>$960K</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -2669,15 +2665,15 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MCH SFR NC OWNER 1 LP LIMITED PARTNERSHIP</t>
+          <t>NOWELL SENIOR TRUST</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Raleigh, Wake Forest</t>
+          <t>Knightdale, Raleigh</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2686,7 +2682,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2695,19 +2691,15 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>$3.6M</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>2021-12</t>
-        </is>
-      </c>
+          <t>$1.3M</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -2717,24 +2709,24 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>MCH SFR NC OWNER 1 LP</t>
+          <t>CHARLES SFR LLC</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Holly Springs, Knightdale, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
@@ -2748,12 +2740,12 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>$8.5M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>2021-12</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
@@ -2765,15 +2757,15 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>SMSLSH LP</t>
+          <t>WONGFRATRIS INVESTMENT COMPANY</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Apex, Cary, Raleigh</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2782,7 +2774,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2791,17 +2783,17 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>$2.2M</t>
+          <t>$2.4M</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -2813,15 +2805,15 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>SMSLSH LP LIMITED PARTNERSHIP</t>
+          <t>WANG, JING</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Apex, Cary</t>
+          <t>Cary, Raleigh</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2830,7 +2822,7 @@
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
@@ -2839,17 +2831,17 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>$2.6M</t>
+          <t>$3.5M</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>2020-07</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -2861,24 +2853,24 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MCH SFR NC OWNER 2 LP</t>
+          <t>THE BLACKBURNS PROJECT LLC</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -2892,12 +2884,12 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>$8.1M</t>
+          <t>$600K</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -2909,7 +2901,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>VOGLER, JAMES BREVARD III TRUSTEE LINDEN, SARAH SKYE TRUSTEE</t>
+          <t>SHELL VILLA LLC</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -2926,7 +2918,7 @@
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
@@ -2935,17 +2927,17 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>$2.0M</t>
+          <t>$1.9M</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>2015-11</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -2957,24 +2949,24 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>CBAR ASSET COMPANY LLC</t>
+          <t>PAL, ANKUR B TRUSTEE PATAN, SUMERA TRUSTEE</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Garner, Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Cary, Fuquay-Varina</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2988,12 +2980,12 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>$3.8M</t>
+          <t>$895K</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3005,24 +2997,24 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>VESTED REALTY LLC</t>
+          <t>DROSSOS, KRISTINA A TRUSTEE KRISTINA A DROSSOS FAMILY TRUST</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Rolesville</t>
+          <t>Fuquay-Varina</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
@@ -3036,12 +3028,12 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>$2.0M</t>
+          <t>$925K</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -3053,11 +3045,11 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SIGNATURE VENTURES PARTNERS LLC</t>
+          <t>TYSOR, CAROL ANN TRUSTEE TYSOR, CAROL ANN TRUSTEE</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
@@ -3070,7 +3062,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3079,19 +3071,15 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>$5.1M</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
+          <t>$1.9M</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -3101,24 +3089,24 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>APOSTLE INC</t>
+          <t>SFR JV-3 PROPERTY LLC</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Raleigh, Rolesville</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
@@ -3132,12 +3120,12 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>$5.0M</t>
+          <t>$703K</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
@@ -3149,24 +3137,24 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PROGRESS RALEIGH LLC</t>
+          <t>MA, WILSON TRUSTEE YEUNG, CHERRI KIN-YEE TRUSTEE</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3180,12 +3168,12 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>$35.0M</t>
+          <t>$722K</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3197,24 +3185,24 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>ARMM ASSETS 2 LLC</t>
+          <t>KULKARNI, ROHAN ANANT TRUSTEE JOSHI, SAI PRADEEP TRUSTEE</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Knightdale, Raleigh, Wendell</t>
+          <t>Apex, Rolesville, Wake Forest</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
@@ -3228,12 +3216,12 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>$4.5M</t>
+          <t>$1.2M</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
@@ -3245,15 +3233,15 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>PROGESS RESIDENTIAL BORROWER 1 LLC</t>
+          <t>TULE RIVER HOMEBUYER EARNED EQUITY AGENCY</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest, Wendell</t>
+          <t>Garner, Raleigh</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3262,7 +3250,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3271,17 +3259,17 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>$2.3M</t>
+          <t>$1.4M</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3293,24 +3281,24 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>KL LB BUY 3 LLC</t>
+          <t>OFFERPAD POINT LLC</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Apex</t>
+          <t>Fuquay-Varina, Raleigh</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
@@ -3324,12 +3312,12 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>$10.2M</t>
+          <t>$777K</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -3341,11 +3329,11 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>HRA U SUITES LLC</t>
+          <t>BLUE C RENTALS NC LLC</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>136</v>
+        <v>2</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
@@ -3354,11 +3342,11 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3372,12 +3360,12 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>$41.5M</t>
+          <t>$680K</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>2015-07</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -3389,15 +3377,15 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>OLYMPUS BORROWER LLC</t>
+          <t>MILLROSE PROPERTIES NORTH CAROLINA, LLC</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3406,7 +3394,7 @@
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
@@ -3420,14 +3408,10 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>$3.8M</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>2022-04</t>
-        </is>
-      </c>
+          <t>$1.0M</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr"/>
       <c r="J61" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -3437,24 +3421,24 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>OLYMPUS BORROWER 1 LLC</t>
+          <t>TRUE REAL ESTATE INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Knightdale, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3468,12 +3452,12 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>$8.6M</t>
+          <t>$795K</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3485,15 +3469,15 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>AO PROPCO 2 LP LIMITED PARTNERSHIP</t>
+          <t>TRUE NORTH PROPERTY OWNER C LLC</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Wendell</t>
+          <t>Fuquay-Varina, Garner, Raleigh</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3502,7 +3486,7 @@
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
@@ -3516,12 +3500,12 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>$3.3M</t>
+          <t>$3.8M</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2023-01</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -3533,15 +3517,15 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>HOME SFR BORROWER LLC</t>
+          <t>DANEBORG NC LLC</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Cary, Fuquay-Varina</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3550,7 +3534,7 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3564,12 +3548,12 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>$1.7M</t>
+          <t>$1.0M</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2022-05</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3581,24 +3565,24 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>TRUE NORTH PROPERTY OWNER B LLC</t>
+          <t>KU, PEI-YU TRUSTEE PEI-YU KU REVOCABLE LIVING TRUST</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Wake Forest</t>
+          <t>Apex, Cary</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
@@ -3612,12 +3596,12 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>$9.2M</t>
+          <t>$1.2M</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -3629,15 +3613,15 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>USCMF MARSHALL PARK LLC</t>
+          <t>DAVIDSON HOMES LLC</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Knightdale, Wake Forest</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3646,7 +3630,7 @@
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3655,19 +3639,15 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>$9.1M</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>2019-02</t>
-        </is>
-      </c>
+          <t>$4.1M</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -3677,24 +3657,24 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>HOME SFR BORROWER IV LLC</t>
+          <t>WAHED FINANCIAL LLC</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Raleigh</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
@@ -3708,12 +3688,12 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>$2.1M</t>
+          <t>$898K</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>2017-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
@@ -3725,24 +3705,24 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>CPI/EV ABODE ALDERWOOD OWNER LLC</t>
+          <t>RESTING PLACE PROPERTIES LLC</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Apex</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3756,12 +3736,12 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>$30.0M</t>
+          <t>$629K</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3773,24 +3753,24 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>STAGE II PROPERTIES LLC</t>
+          <t>GANGARAPU, SHASHIKANTH TRUSTEE MAMILLA, TEJASWI TRUSTEE</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Garner, Raleigh, Wendell</t>
+          <t>Cary, Rolesville</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
@@ -3804,12 +3784,12 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>$1.9M</t>
+          <t>$918K</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>2017-08</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -3821,15 +3801,15 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>CANNON NC RENTALS LLC</t>
+          <t>SRAM PACK I-C LLC</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Garner, Knightdale, Raleigh, Wendell</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3838,7 +3818,7 @@
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3852,12 +3832,12 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>$2.8M</t>
+          <t>$2.9M</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2022-08</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3869,24 +3849,24 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>AMH ROMAN TWO NC LLC</t>
+          <t>PLUTUS ESTATES LLC</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Apex, Cary, Fuquay-Varina, Raleigh, Wake Forest</t>
+          <t>Garner, Wendell</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
@@ -3900,12 +3880,12 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>$5.9M</t>
+          <t>$720K</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>2016-03</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
@@ -3917,24 +3897,24 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>THE CIANO FAMILY TRUST</t>
+          <t>LITTLE, YVONNE TRUSTEE YVONNE LITTLE TRUST</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest</t>
+          <t>Garner, Raleigh</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3948,12 +3928,12 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>$1.4M</t>
+          <t>$707K</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>2021-06</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3965,24 +3945,24 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>ALTO ASSET COMPANY 3 LLC</t>
+          <t>GUNDA, SRINIVAS TRUSTEE GANDE, KAVITHA TRUSTEE</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh, Rolesville</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
@@ -3996,12 +3976,12 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>$5.4M</t>
+          <t>$649K</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>2020-04</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
@@ -4013,24 +3993,24 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>THE TRUST OF BOONE WAKE COUNTY NORTH CAROLINA WCNC</t>
+          <t>A&amp;N HOUSING LLC</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Wake Forest</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4039,17 +4019,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>$2.4M</t>
+          <t>$773K</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-10</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4061,15 +4041,15 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>ALVAR NC LLC</t>
+          <t>GE, DONGLIANG LIU, LI</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Cary, Raleigh, Wendell</t>
+          <t>Cary, Garner, Holly Springs</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -4078,7 +4058,7 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
@@ -4087,17 +4067,17 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>$33.3M</t>
+          <t>$2.5M</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>2018-05</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
@@ -4109,15 +4089,15 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>SAFARI TWO ASSET COMPANY LLC</t>
+          <t>CARUSO BUILDER WENDELL FALLS LLC</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest</t>
+          <t>Wendell</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -4126,7 +4106,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4140,14 +4120,10 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>$5.6M</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>2018-06</t>
-        </is>
-      </c>
+          <t>$1.9M</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -4157,24 +4133,24 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>SAFARI ONE ASSET COMPANY, LLC</t>
+          <t>KGC INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest</t>
+          <t>Wendell</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
@@ -4188,12 +4164,12 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>$1.7M</t>
+          <t>$589K</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>2017-08</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
@@ -4205,11 +4181,11 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>SAFARI ONE ASSET COMPANY LLC</t>
+          <t>VP PARADE LLC</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
@@ -4218,11 +4194,11 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4236,12 +4212,12 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>$2.7M</t>
+          <t>$840K</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>2018-06</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4253,24 +4229,24 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>BBRK LLC</t>
+          <t>MAS CAPITAL VENTURES LLC</t>
         </is>
       </c>
       <c r="B79" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Apex, Cary, Holly Springs, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
@@ -4279,17 +4255,17 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>$2.6M</t>
+          <t>$2.2M</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>2020-05</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
@@ -4301,24 +4277,24 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES, L.P., LIMITED PARTNERSHIP</t>
+          <t>LEESVILLE BLUE HOLDINGS LLC</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4327,17 +4303,17 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>$4.8M</t>
+          <t>$1.0M</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>2017-12</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4349,24 +4325,24 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>HEBERT, ERIC TRUSTEE THE ERIC HEBERT FAMILY TRUST</t>
+          <t>660 DFH II LLC</t>
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Cary, Fuquay-Varina</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
@@ -4375,17 +4351,17 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>$3.4M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>2016-12</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
@@ -4397,24 +4373,24 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES, L.P.</t>
+          <t>FOREVER P&amp;T REALTY LLC</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Rolesville, Wake Forest</t>
+          <t>Cary, Holly Springs</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4423,17 +4399,17 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>$3.4M</t>
+          <t>$2.5M</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -4445,24 +4421,24 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES TWO LP LIMITED PARTNERSHIP</t>
+          <t>NC 3116 HILLSBOROUGH LLC</t>
         </is>
       </c>
       <c r="B83" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
@@ -4471,17 +4447,17 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 500K 1M; Absentee Out Of State; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>$2.5M</t>
+          <t>$1.5M</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
@@ -4493,24 +4469,24 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>RXR LEN APEX OWNER LLC</t>
+          <t>HSU, WILLIE TRUSTEE CHEN, SHIH CHEN TRUSTEE</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Apex</t>
+          <t>Apex, Cary</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4524,12 +4500,12 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>$3.3M</t>
+          <t>$957K</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2021-12</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4541,24 +4517,24 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>NOBLE-CARBAJAL, MELADEE TRUSTEE MELADEE NOBLE 2019 TRUST</t>
+          <t>STRASZEWSKI, EDWARD R TRUSTEE STRASZEWSKI, MARY M TRUSTEE</t>
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
@@ -4572,12 +4548,12 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>$909K</t>
+          <t>$920K</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>2020-08</t>
+          <t>2021-05</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
@@ -4589,24 +4565,24 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES TWO LP</t>
+          <t>GILADI INVESTMENTS LLC</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -4620,12 +4596,12 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>$10.1M</t>
+          <t>$994K</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2019-12</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4637,15 +4613,15 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>ALTO ASSET COMPANY 1 LLC</t>
+          <t>SFKG LLC</t>
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Knightdale, Raleigh</t>
+          <t>Wendell</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4654,7 +4630,7 @@
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
@@ -4663,17 +4639,17 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Llc Corp Owned; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>$2.3M</t>
+          <t>$2.2M</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>2019-12</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
@@ -4685,24 +4661,24 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES LP LIMITED PARTNERSHIP</t>
+          <t>STOKES, KATHERINE FULLER TRUSTEE THE KATHERINE FULLER STOKES REVOCABLE DECLARATION</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Cary, Fuquay-Varina, Garner, Holly Springs, Raleigh, Rolesville, Wake Forest</t>
+          <t>Raleigh, Wake Forest</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -4716,12 +4692,12 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>$10.9M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>2017-10</t>
+          <t>2013-06</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4733,24 +4709,24 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>AMH NC PROPERTIES LP</t>
+          <t>LANG, DAVID H TRUSTEE LAMPERT, CHRISTINE M TRUSTEE</t>
         </is>
       </c>
       <c r="B89" s="3" t="n">
-        <v>149</v>
+        <v>2</v>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Rolesville, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
@@ -4764,12 +4740,12 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>$57.0M</t>
+          <t>$966K</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2005-07</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
@@ -4781,24 +4757,24 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>21 JUMPSTREET LLC</t>
+          <t>DMBE PROPERTIES LLC</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Fuquay-Varina</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Foreign National Investor</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -4807,17 +4783,17 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Foreign Owner; Llc Corp Owned</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>$1.7M</t>
+          <t>$717K</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>2012-11</t>
+          <t>2012-02</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -4829,24 +4805,24 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>RS RENTAL III-B LLC</t>
+          <t>HUANG ESTATES LLC</t>
         </is>
       </c>
       <c r="B91" s="3" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Raleigh, Wake Forest, Wendell</t>
+          <t>Apex, Cary</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
@@ -4860,12 +4836,12 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>$4.3M</t>
+          <t>$988K</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2021-08</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
@@ -4877,24 +4853,24 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>RS RENTAL II LLC</t>
+          <t>SOUTHERN PEONY, LLC</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Garner, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -4908,12 +4884,12 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>$10.9M</t>
+          <t>$667K</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>2021-12</t>
+          <t>2016-08</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4925,11 +4901,11 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>PATRIOT CANYON PROPERTIES LLC</t>
+          <t>BZRE LLC</t>
         </is>
       </c>
       <c r="B93" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
@@ -4938,11 +4914,11 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
@@ -4956,12 +4932,12 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>$1.7M</t>
+          <t>$1.0M</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>2016-06</t>
+          <t>2019-05</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
@@ -4973,24 +4949,24 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>AMH 2015-2 BORROWER LP LIMITED PARTNERSHIP</t>
+          <t>SOPKO, EMILY TRUSTEE SOPKO, KYLE TRUSTEE</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Garner, Holly Springs, Raleigh, Rolesville, Wake Forest</t>
+          <t>Cary, Holly Springs</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5004,12 +4980,12 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>$15.1M</t>
+          <t>$784K</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2020-09</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -5021,15 +4997,15 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>RS RENTAL I LLC</t>
+          <t>HOUSTON, CHRISTOPHER</t>
         </is>
       </c>
       <c r="B95" s="3" t="n">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Garner, Holly Springs, Knightdale, Raleigh, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -5038,7 +5014,7 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
@@ -5047,17 +5023,17 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>$17.9M</t>
+          <t>$1.3M</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2006-01</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
@@ -5069,24 +5045,24 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AMH 2015-2 BORROWER LLC</t>
+          <t>NYC NORTH LLC</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>189</v>
+        <v>4</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Apex, Cary, Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Rolesville, Wake Forest</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5100,12 +5076,12 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>$67.8M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>2015-03</t>
+          <t>2014-05</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5117,24 +5093,24 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>AMH 2015-1 BORROWER LLC</t>
+          <t>PLANIT PROPERTIES LLC</t>
         </is>
       </c>
       <c r="B97" s="3" t="n">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Apex, Cary, Fuquay-Varina, Garner, Holly Springs, Raleigh, Wake Forest, Wendell</t>
+          <t>Cary, Raleigh</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
@@ -5148,12 +5124,12 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>$37.1M</t>
+          <t>$915K</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>2014-09</t>
+          <t>2005-07</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
@@ -5165,15 +5141,15 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>AMH 2014-3 BORROWER LP</t>
+          <t>DUKES PROPERTIES &amp; CONSTRUCTION LLC</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Garner, Holly Springs, Knightdale, Raleigh</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5182,7 +5158,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5191,17 +5167,17 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Llc Corp Owned; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>$5.5M</t>
+          <t>$3.3M</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>2016-03</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5213,24 +5189,24 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>ZOOMZ INVESTMENTS LLC</t>
+          <t>NOBLE, JANAE TRUSTEE JANAE NOBLE TRUST</t>
         </is>
       </c>
       <c r="B99" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Apex, Fuquay-Varina, Wendell</t>
+          <t>Garner, Wake Forest</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
@@ -5244,12 +5220,12 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>$1.5M</t>
+          <t>$631K</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>2021-05</t>
+          <t>2017-08</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
@@ -5261,15 +5237,15 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>AMH 2014-3 BORROWER LLC</t>
+          <t>THEISS, DAVID V</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
-        <v>263</v>
+        <v>5</v>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Apex, Cary, Fuquay-Varina, Garner, Holly Springs, Knightdale, Raleigh, Rolesville, Wake Forest, Wendell</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -5278,7 +5254,7 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5287,17 +5263,17 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Llc Corp Owned</t>
+          <t>No Homestead; Value 150K 500K; Absentee Out Of State; Portfolio 5 Plus</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>$96.1M</t>
+          <t>$1.5M</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>2014-03</t>
+          <t>2007-06</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -5309,24 +5285,24 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>ALTO ASSET COMPANY 2 LLC</t>
+          <t>HOPEG TRADING LLC</t>
         </is>
       </c>
       <c r="B101" s="3" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Fuquay-Varina, Raleigh, Wake Forest</t>
+          <t>Apex, Fuquay-Varina, Holly Springs</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Landlord (5+)</t>
+          <t>Out-of-State Investor</t>
         </is>
       </c>
       <c r="E101" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
@@ -5340,12 +5316,12 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>$5.1M</t>
+          <t>$1.1M</t>
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>2020-03</t>
+          <t>2021-03</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr">

</xml_diff>